<commit_message>
melhorias graficas e site map
</commit_message>
<xml_diff>
--- a/operation_log.xlsx
+++ b/operation_log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1560"/>
+  <dimension ref="A1:O1563"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -73719,9 +73719,150 @@
         <v>1</v>
       </c>
     </row>
+    <row r="1561">
+      <c r="A1561" t="str">
+        <v>2025-04-09T13:08:44.268Z</v>
+      </c>
+      <c r="B1561" t="str">
+        <v>123456</v>
+      </c>
+      <c r="C1561" t="b">
+        <v>1</v>
+      </c>
+      <c r="D1561" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1561" t="b">
+        <v>1</v>
+      </c>
+      <c r="F1561" t="b">
+        <v>1</v>
+      </c>
+      <c r="G1561" t="b">
+        <v>1</v>
+      </c>
+      <c r="H1561" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1561">
+        <v>0</v>
+      </c>
+      <c r="J1561">
+        <v>0</v>
+      </c>
+      <c r="K1561" t="str">
+        <v>25</v>
+      </c>
+      <c r="L1561" t="str">
+        <v>0</v>
+      </c>
+      <c r="M1561" t="str">
+        <v>0</v>
+      </c>
+      <c r="N1561" t="str">
+        <v>0</v>
+      </c>
+      <c r="O1561" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" t="str">
+        <v>2025-04-09T13:08:45.958Z</v>
+      </c>
+      <c r="B1562" t="str">
+        <v>123456</v>
+      </c>
+      <c r="C1562" t="b">
+        <v>1</v>
+      </c>
+      <c r="D1562" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1562" t="b">
+        <v>1</v>
+      </c>
+      <c r="F1562" t="b">
+        <v>1</v>
+      </c>
+      <c r="G1562" t="b">
+        <v>1</v>
+      </c>
+      <c r="H1562" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1562">
+        <v>0</v>
+      </c>
+      <c r="J1562">
+        <v>0</v>
+      </c>
+      <c r="K1562" t="str">
+        <v>25</v>
+      </c>
+      <c r="L1562" t="str">
+        <v>0</v>
+      </c>
+      <c r="M1562" t="str">
+        <v>0</v>
+      </c>
+      <c r="N1562" t="str">
+        <v>0</v>
+      </c>
+      <c r="O1562" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" t="str">
+        <v>2025-04-09T13:08:49.282Z</v>
+      </c>
+      <c r="B1563" t="str">
+        <v>123456</v>
+      </c>
+      <c r="C1563" t="b">
+        <v>1</v>
+      </c>
+      <c r="D1563" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1563" t="b">
+        <v>1</v>
+      </c>
+      <c r="F1563" t="b">
+        <v>1</v>
+      </c>
+      <c r="G1563" t="b">
+        <v>1</v>
+      </c>
+      <c r="H1563" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1563">
+        <v>0</v>
+      </c>
+      <c r="J1563">
+        <v>0</v>
+      </c>
+      <c r="K1563" t="str">
+        <v>25</v>
+      </c>
+      <c r="L1563" t="str">
+        <v>0</v>
+      </c>
+      <c r="M1563" t="str">
+        <v>0</v>
+      </c>
+      <c r="N1563" t="str">
+        <v>0</v>
+      </c>
+      <c r="O1563" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O1560"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1563"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
corrigido travamnto do carrinho quando o sistema fisico acaba o trecho antes (buffer de 1)
</commit_message>
<xml_diff>
--- a/operation_log.xlsx
+++ b/operation_log.xlsx
@@ -413,7 +413,7 @@
         <v>Início</v>
       </c>
       <c r="B2" t="str">
-        <v>2025-07-02T14:57:13.696Z</v>
+        <v>2025-07-02T16:20:24.875Z</v>
       </c>
     </row>
     <row r="3">
@@ -433,7 +433,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -481,7 +481,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-07-02T14:57:13.807Z</v>
+        <v>2025-07-02T16:20:25.005Z</v>
       </c>
       <c r="B2" t="b">
         <v>1</v>
@@ -493,13 +493,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -508,16 +508,16 @@
         <v>0</v>
       </c>
       <c r="J2" t="str">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="K2" t="str">
-        <v>1931</v>
+        <v>5614</v>
       </c>
       <c r="L2" t="str">
-        <v>-30.07</v>
+        <v>-19.91</v>
       </c>
       <c r="M2" t="str">
-        <v>3.99</v>
+        <v>4.15</v>
       </c>
       <c r="N2" t="b">
         <v>0</v>
@@ -525,10 +525,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-07-02T14:57:17.352Z</v>
+        <v>2025-07-02T16:20:25.580Z</v>
       </c>
       <c r="B3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -537,13 +537,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -552,16 +552,16 @@
         <v>0</v>
       </c>
       <c r="J3" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K3" t="str">
-        <v>1941</v>
+        <v>5614</v>
       </c>
       <c r="L3" t="str">
-        <v>-30.07</v>
+        <v>-19.91</v>
       </c>
       <c r="M3" t="str">
-        <v>4</v>
+        <v>4.15</v>
       </c>
       <c r="N3" t="b">
         <v>0</v>
@@ -569,7 +569,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-07-02T14:57:29.355Z</v>
+        <v>2025-07-02T16:20:31.627Z</v>
       </c>
       <c r="B4" t="b">
         <v>0</v>
@@ -581,16 +581,16 @@
         <v>1</v>
       </c>
       <c r="E4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -599,13 +599,13 @@
         <v>25</v>
       </c>
       <c r="K4" t="str">
-        <v>1952</v>
+        <v>5614</v>
       </c>
       <c r="L4" t="str">
-        <v>-28.76</v>
+        <v>-19.91</v>
       </c>
       <c r="M4" t="str">
-        <v>3.96</v>
+        <v>4.15</v>
       </c>
       <c r="N4" t="b">
         <v>0</v>
@@ -613,7 +613,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2025-07-02T14:57:37.347Z</v>
+        <v>2025-07-02T16:20:38.658Z</v>
       </c>
       <c r="B5" t="b">
         <v>1</v>
@@ -625,16 +625,16 @@
         <v>1</v>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -643,13 +643,13 @@
         <v>25</v>
       </c>
       <c r="K5" t="str">
-        <v>1962</v>
+        <v>5614</v>
       </c>
       <c r="L5" t="str">
-        <v>-27.9</v>
+        <v>-19.91</v>
       </c>
       <c r="M5" t="str">
-        <v>3.96</v>
+        <v>4.15</v>
       </c>
       <c r="N5" t="b">
         <v>0</v>
@@ -657,7 +657,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-07-02T14:57:39.474Z</v>
+        <v>2025-07-02T17:36:42.444Z</v>
       </c>
       <c r="B6" t="b">
         <v>1</v>
@@ -666,7 +666,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -675,25 +675,25 @@
         <v>1</v>
       </c>
       <c r="G6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K6" t="str">
-        <v>1962</v>
+        <v>4183</v>
       </c>
       <c r="L6" t="str">
-        <v>-27.9</v>
+        <v>0</v>
       </c>
       <c r="M6" t="str">
-        <v>3.96</v>
+        <v>4.18</v>
       </c>
       <c r="N6" t="b">
         <v>0</v>
@@ -701,7 +701,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-07-02T14:57:45.479Z</v>
+        <v>2025-07-02T17:36:44.344Z</v>
       </c>
       <c r="B7" t="b">
         <v>1</v>
@@ -713,31 +713,31 @@
         <v>1</v>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K7" t="str">
-        <v>1972</v>
+        <v>4193</v>
       </c>
       <c r="L7" t="str">
-        <v>-25.52</v>
+        <v>0</v>
       </c>
       <c r="M7" t="str">
-        <v>3.96</v>
+        <v>4.18</v>
       </c>
       <c r="N7" t="b">
         <v>0</v>
@@ -745,7 +745,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-07-02T14:57:51.559Z</v>
+        <v>2025-07-02T17:36:45.272Z</v>
       </c>
       <c r="B8" t="b">
         <v>1</v>
@@ -757,31 +757,31 @@
         <v>1</v>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K8" t="str">
-        <v>1972</v>
+        <v>4193</v>
       </c>
       <c r="L8" t="str">
-        <v>-25.52</v>
+        <v>0</v>
       </c>
       <c r="M8" t="str">
-        <v>3.96</v>
+        <v>4.18</v>
       </c>
       <c r="N8" t="b">
         <v>0</v>
@@ -789,10 +789,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2025-07-02T14:58:12.631Z</v>
+        <v>2025-07-02T17:36:57.467Z</v>
       </c>
       <c r="B9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -807,25 +807,25 @@
         <v>1</v>
       </c>
       <c r="G9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K9" t="str">
-        <v>1993</v>
+        <v>4204</v>
       </c>
       <c r="L9" t="str">
-        <v>-22.83</v>
+        <v>0</v>
       </c>
       <c r="M9" t="str">
-        <v>3.94</v>
+        <v>4.18</v>
       </c>
       <c r="N9" t="b">
         <v>0</v>
@@ -833,43 +833,43 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2025-07-02T14:58:13.671Z</v>
+        <v>2025-07-02T17:37:05.590Z</v>
       </c>
       <c r="B10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
       </c>
       <c r="D10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
       </c>
       <c r="F10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K10" t="str">
-        <v>1993</v>
+        <v>4214</v>
       </c>
       <c r="L10" t="str">
-        <v>-22.83</v>
+        <v>0</v>
       </c>
       <c r="M10" t="str">
-        <v>3.94</v>
+        <v>4.18</v>
       </c>
       <c r="N10" t="b">
         <v>0</v>
@@ -877,10 +877,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2025-07-02T14:58:24.633Z</v>
+        <v>2025-07-02T17:37:16.022Z</v>
       </c>
       <c r="B11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
@@ -892,28 +892,28 @@
         <v>1</v>
       </c>
       <c r="F11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K11" t="str">
-        <v>2003</v>
+        <v>4224</v>
       </c>
       <c r="L11" t="str">
-        <v>-21.48</v>
+        <v>0</v>
       </c>
       <c r="M11" t="str">
-        <v>3.95</v>
+        <v>4.18</v>
       </c>
       <c r="N11" t="b">
         <v>0</v>
@@ -921,7 +921,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2025-07-02T14:58:26.714Z</v>
+        <v>2025-07-02T17:37:19.708Z</v>
       </c>
       <c r="B12" t="b">
         <v>1</v>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="G12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -951,13 +951,13 @@
         <v>0</v>
       </c>
       <c r="K12" t="str">
-        <v>2013</v>
+        <v>4224</v>
       </c>
       <c r="L12" t="str">
-        <v>-19.96</v>
+        <v>0</v>
       </c>
       <c r="M12" t="str">
-        <v>3.98</v>
+        <v>4.18</v>
       </c>
       <c r="N12" t="b">
         <v>0</v>
@@ -965,10 +965,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2025-07-02T15:07:24.041Z</v>
+        <v>2025-07-02T17:37:32.847Z</v>
       </c>
       <c r="B13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" t="b">
         <v>1</v>
@@ -995,13 +995,13 @@
         <v>0</v>
       </c>
       <c r="K13" t="str">
-        <v>2545</v>
+        <v>4234</v>
       </c>
       <c r="L13" t="str">
-        <v>-19.96</v>
+        <v>0.02</v>
       </c>
       <c r="M13" t="str">
-        <v>4.18</v>
+        <v>4.2</v>
       </c>
       <c r="N13" t="b">
         <v>0</v>
@@ -1009,7 +1009,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2025-07-02T15:08:11.042Z</v>
+        <v>2025-07-02T17:37:36.576Z</v>
       </c>
       <c r="B14" t="b">
         <v>1</v>
@@ -1039,21 +1039,329 @@
         <v>0</v>
       </c>
       <c r="K14" t="str">
-        <v>2596</v>
+        <v>4244</v>
       </c>
       <c r="L14" t="str">
-        <v>-19.96</v>
+        <v>0.02</v>
       </c>
       <c r="M14" t="str">
-        <v>4.18</v>
+        <v>4.2</v>
       </c>
       <c r="N14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2025-07-02T17:37:46.577Z</v>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15" t="str">
+        <v>0</v>
+      </c>
+      <c r="K15" t="str">
+        <v>4254</v>
+      </c>
+      <c r="L15" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="M15" t="str">
+        <v>4.2</v>
+      </c>
+      <c r="N15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2025-07-02T17:38:11.280Z</v>
+      </c>
+      <c r="B16" t="b">
+        <v>1</v>
+      </c>
+      <c r="C16" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="b">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16" t="str">
+        <v>0</v>
+      </c>
+      <c r="K16" t="str">
+        <v>4275</v>
+      </c>
+      <c r="L16" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="M16" t="str">
+        <v>4.2</v>
+      </c>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2025-07-02T17:38:14.555Z</v>
+      </c>
+      <c r="B17" t="b">
+        <v>1</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17" t="str">
+        <v>0</v>
+      </c>
+      <c r="K17" t="str">
+        <v>4275</v>
+      </c>
+      <c r="L17" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="M17" t="str">
+        <v>4.2</v>
+      </c>
+      <c r="N17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2025-07-02T17:38:27.760Z</v>
+      </c>
+      <c r="B18" t="b">
+        <v>1</v>
+      </c>
+      <c r="C18" t="b">
+        <v>1</v>
+      </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" t="b">
+        <v>1</v>
+      </c>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18" t="str">
+        <v>0</v>
+      </c>
+      <c r="K18" t="str">
+        <v>4295</v>
+      </c>
+      <c r="L18" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="M18" t="str">
+        <v>4.2</v>
+      </c>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2025-07-02T17:38:30.361Z</v>
+      </c>
+      <c r="B19" t="b">
+        <v>1</v>
+      </c>
+      <c r="C19" t="b">
+        <v>1</v>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" t="b">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19" t="str">
+        <v>0</v>
+      </c>
+      <c r="K19" t="str">
+        <v>4295</v>
+      </c>
+      <c r="L19" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="M19" t="str">
+        <v>4.2</v>
+      </c>
+      <c r="N19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2025-07-02T17:38:39.935Z</v>
+      </c>
+      <c r="B20" t="b">
+        <v>1</v>
+      </c>
+      <c r="C20" t="b">
+        <v>1</v>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" t="b">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20" t="str">
+        <v>0</v>
+      </c>
+      <c r="K20" t="str">
+        <v>4305</v>
+      </c>
+      <c r="L20" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="M20" t="str">
+        <v>4.2</v>
+      </c>
+      <c r="N20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2025-07-02T17:38:45.348Z</v>
+      </c>
+      <c r="B21" t="b">
+        <v>1</v>
+      </c>
+      <c r="C21" t="b">
+        <v>1</v>
+      </c>
+      <c r="D21" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="b">
+        <v>1</v>
+      </c>
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21" t="str">
+        <v>0</v>
+      </c>
+      <c r="K21" t="str">
+        <v>4316</v>
+      </c>
+      <c r="L21" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="M21" t="str">
+        <v>4.2</v>
+      </c>
+      <c r="N21" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajustes de angulo camera
</commit_message>
<xml_diff>
--- a/operation_log.xlsx
+++ b/operation_log.xlsx
@@ -433,7 +433,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1359,9 +1359,185 @@
         <v>0</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2025-07-02T17:53:35.837Z</v>
+      </c>
+      <c r="B22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C22" t="b">
+        <v>1</v>
+      </c>
+      <c r="D22" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" t="b">
+        <v>1</v>
+      </c>
+      <c r="G22" t="b">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>5</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22" t="str">
+        <v>0</v>
+      </c>
+      <c r="K22" t="str">
+        <v>5201</v>
+      </c>
+      <c r="L22" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="M22" t="str">
+        <v>4.19</v>
+      </c>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2025-07-02T17:53:38.851Z</v>
+      </c>
+      <c r="B23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>6</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23" t="str">
+        <v>0</v>
+      </c>
+      <c r="K23" t="str">
+        <v>5201</v>
+      </c>
+      <c r="L23" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="M23" t="str">
+        <v>4.19</v>
+      </c>
+      <c r="N23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2025-07-02T17:53:49.902Z</v>
+      </c>
+      <c r="B24" t="b">
+        <v>1</v>
+      </c>
+      <c r="C24" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" t="b">
+        <v>1</v>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" t="b">
+        <v>1</v>
+      </c>
+      <c r="G24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>15</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24" t="str">
+        <v>0</v>
+      </c>
+      <c r="K24" t="str">
+        <v>5211</v>
+      </c>
+      <c r="L24" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="M24" t="str">
+        <v>4.19</v>
+      </c>
+      <c r="N24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2025-07-02T17:54:00.958Z</v>
+      </c>
+      <c r="B25" t="b">
+        <v>1</v>
+      </c>
+      <c r="C25" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" t="b">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>29</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25" t="str">
+        <v>0</v>
+      </c>
+      <c r="K25" t="str">
+        <v>5232</v>
+      </c>
+      <c r="L25" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="M25" t="str">
+        <v>4.19</v>
+      </c>
+      <c r="N25" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>